<commit_message>
fix: grupos.xlsx - novos nomes do Sonda (Lager Heineken 350ml, Michelob garrafa 330ml) e grupo errado do Heineken 269ml
</commit_message>
<xml_diff>
--- a/grupos.xlsx
+++ b/grupos.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilha1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="82.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cerveja Lager Zero Álcool Heineken Lata 350ml</t>
+          <t>Cerveja Lager Heineken 350ml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -662,19 +662,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>6.81</v>
+      <c r="D6" t="n">
+        <v>4.79</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Heineken 0% 350ml</t>
+          <t>Heineken 350ml</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cerveja 0,0% álcool Heineken long neck 330ml</t>
+          <t>Cerveja Lager Zero Álcool Heineken Lata 350ml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -688,18 +688,18 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8.02</v>
+        <v>6.81</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Heineken 0% 330ml LN</t>
+          <t>Heineken 0% 350ml</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cerveja Heineken long neck 330ml</t>
+          <t>Cerveja 0,0% álcool Heineken long neck 330ml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -717,14 +717,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Heineken LN 330ml</t>
+          <t>Heineken 0% 330ml LN</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cerveja Lager Puro Malte sem Glúten Heineken Ultimate Garrafa 330ml</t>
+          <t>Cerveja Heineken long neck 330ml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -742,14 +742,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Heineken Ultimate 330ml</t>
+          <t>Heineken LN 330ml</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cerveja Heineken Lata - 473ml</t>
+          <t>Cerveja Lager Puro Malte sem Glúten Heineken Ultimate Garrafa 330ml</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -763,57 +763,57 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>8.130000000000001</v>
+        <v>8.02</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Heineken latão</t>
+          <t>Heineken Ultimate 330ml</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cerveja Lager Heineken Garrafa 600ml</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>13.48</v>
+          <t>Cerveja Heineken Lata - 473ml</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>8.130000000000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Heineken Garrafa 600 ml</t>
+          <t>Heineken latão</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cerveja Heineken long neck 600ml</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Cerveja Lager Heineken Garrafa 600ml</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>13.48</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>15.28</v>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -824,126 +824,126 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Cerveja Heineken long neck 600ml</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>15.28</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Heineken Garrafa 600 ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Cerveja Heineken Long Neck 6x250ml</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B14" s="6" t="n">
         <v>31.98</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C14" s="6" t="n">
         <v>5.33</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Heineken LN 250 ml</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="C14" t="inlineStr">
+    <row r="15">
+      <c r="C15" t="inlineStr">
         <is>
           <t>(6 un)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Cerveja Heineken Pack 8 Latas 269ml Cada</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B16" s="6" t="n">
         <v>36.98</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C16" s="6" t="n">
         <v>4.62</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Heineken 0% 269</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Heineken 269ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr">
         <is>
           <t>(8 un)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Cerveja Heineken Zero Álcool Pack 8 Latas 269ml Cada</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B18" s="6" t="n">
         <v>36.98</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>4.62</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Heineken 0% 269ml</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="C18" t="inlineStr">
+    <row r="19">
+      <c r="C19" t="inlineStr">
         <is>
           <t>(8 un)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Cerveja Lager Premium Puro Malte Zero Álcool Heineken Pack com 6 Unidades 330ml Cada</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>39.98</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Heineken 0% 330ml LN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cerveja Lager Heineken Pack 6 Long Neck 330ml cada</t>
+          <t>Cerveja Lager Premium Puro Malte Zero Álcool Heineken Pack com 6 Unidades 330ml Cada</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>41.98</v>
+        <v>39.98</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -957,143 +957,143 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Heineken LN 330ml</t>
+          <t>Heineken 0% 330ml LN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Cerveja Lager Heineken Pack 6 Long Neck 330ml cada</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Heineken LN 330ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Cerveja Heineken Ultimate Long Neck 6x330ml</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n">
+      <c r="B22" s="6" t="n">
         <v>43.74</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C22" s="6" t="n">
         <v>7.29</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Heineken Ultimate 330ml</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="C22" t="inlineStr">
+    <row r="23">
+      <c r="C23" t="inlineStr">
         <is>
           <t>(6 un)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Cerveja Heineken Sleek Pack 12 Latas 350ml Cada</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B24" s="6" t="n">
         <v>68.48</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C24" s="6" t="n">
         <v>5.71</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Heineken 350ml</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="C24" t="inlineStr">
+    <row r="25">
+      <c r="C25" t="inlineStr">
         <is>
           <t>(12 un)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Cerveja Heineken Zero Álcool Sleek Pack 12 Latas 350ml Cada</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n">
+      <c r="B26" s="6" t="n">
         <v>68.48</v>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C26" s="6" t="n">
         <v>5.71</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Heineken 0% 350ml</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="C26" t="inlineStr">
+    <row r="27">
+      <c r="C27" t="inlineStr">
         <is>
           <t>(12 un)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Cerveja Lager Chopp Premium Heineken Barril 5l</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>109.98</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Barril 5l</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cerveja Heineken barril 5 Litros</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Cerveja Lager Chopp Premium Heineken Barril 5l</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>109.98</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>132.21</v>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1104,86 +1104,86 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chopeira Elétrica Heineken Krups Beertender B101 127V 5l</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>999.9</v>
+          <t>Cerveja Heineken barril 5 Litros</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>132.21</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Chopeira</t>
+          <t>Barril 5l</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Spaten</t>
+          <t>Chopeira Elétrica Heineken Krups Beertender B101 127V 5l</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>999.9</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Chopeira</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Sam's Club</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Sams/un</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Sonda Delivery</t>
+          <t>Spaten</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cerveja munich helles Spaten lata 269ml</t>
+          <t>Produto</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sam's Club</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>3.79</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Spaten lata 269ml</t>
+          <t>Sams/un</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Sonda Delivery</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cerveja munich puro malte Spaten lata 350ml</t>
+          <t>Cerveja munich helles Spaten lata 269ml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1197,18 +1197,18 @@
         </is>
       </c>
       <c r="D33" s="6" t="n">
-        <v>4.89</v>
+        <v>3.79</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Spaten lata 350ml</t>
+          <t>Spaten lata 269ml</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cerveja puro malte Spaten long neck 330ml</t>
+          <t>Cerveja munich puro malte Spaten lata 350ml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1222,57 +1222,57 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>5.99</v>
+        <v>4.89</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Spaten LN</t>
+          <t>Spaten lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cerveja Munich Helles Puro Malte Spaten Garrafa 600ml</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n">
-        <v>9.98</v>
+          <t>Cerveja puro malte Spaten long neck 330ml</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>5.99</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Spaten garrafa 600ml</t>
+          <t>Spaten LN</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cerveja puro malte munich helles Spaten garrafa 600ml</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Cerveja Munich Helles Puro Malte Spaten Garrafa 600ml</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>9.98</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="n">
-        <v>9.99</v>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1283,269 +1283,295 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cerveja puro malte munich helles Spaten garrafa 600ml</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Spaten garrafa 600ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Cerveja Spaten Munich Puro Malte Pack 8 Latas 269ml Cada</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n">
+      <c r="B38" s="6" t="n">
         <v>28.98</v>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C38" s="6" t="n">
         <v>3.62</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>Spaten lata 269ml</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="C38" t="inlineStr">
+    <row r="39">
+      <c r="C39" t="inlineStr">
         <is>
           <t>(8 un)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Cerveja Puro Malte Spaten Munich Pack 12 Unidades de 350ml Cada</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>unit.</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Spaten lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Michelob</t>
+          <t>Cerveja Puro Malte Spaten Munich Pack 12 Unidades de 350ml Cada</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>46.98</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>unit.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Spaten lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Sam's Club</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Sams/un</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Sonda Delivery</t>
+          <t>Michelob</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cerveja ultra Michelob lata 350ml</t>
+          <t>Produto</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sam's Club</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="n">
-        <v>5.82</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Michelob Lata 350 ml</t>
+          <t>Sams/un</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Sonda Delivery</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Cerveja ultra Michelob lata 350ml</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Michelob Lata 350 ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cerveja superior light beer Michelob Ultra garrafa 330ml</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Michelob LN 330ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26.25" customHeight="1" thickBot="1">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Cerveja Michelob Ultra Pack 6 Garrafas 330ml Cada</t>
         </is>
       </c>
-      <c r="B43" s="6" t="n">
+      <c r="B45" s="6" t="n">
         <v>32.94</v>
       </c>
-      <c r="C43" s="6" t="n">
+      <c r="C45" s="6" t="n">
         <v>5.49</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>Michelob LN 330ml</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="C44" t="inlineStr">
+    <row r="46" ht="26.25" customHeight="1" thickBot="1">
+      <c r="C46" t="inlineStr">
         <is>
           <t>(6 un)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Cerveja pure gold Stella Artois lata 269ml</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="n">
-        <v>5.05</v>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Pure Gold lata 269ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Cerveja pure gold Stella Artois lata 350ml</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="n">
-        <v>5.29</v>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Pure Gold lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="47" ht="26.25" customHeight="1" thickBot="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>Cerveja pure gold Stella Artois lata 269ml</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Pure Gold lata 269ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Cerveja pure gold Stella Artois lata 350ml</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Pure Gold lata 350ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>Cerveja pure gold Stella Artois long neck 330ml</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="n">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>7.39</v>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Pure Gold LN 330ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Cerveja Puro Malte Pure Gold sem Glúten Stella Artois Lata 8x269ml</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Pure Gold lata 269ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Cerveja Puro Malte Pure Gold Stella Artois Lata 8x350ml</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Pure Gold lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cerveja Stella Artois Gold Pack 6 Long Neck 330ml Cada</t>
+          <t>Cerveja Puro Malte Pure Gold sem Glúten Stella Artois Lata 8x269ml</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Stella LN 330ml</t>
+          <t>Pure Gold lata 269ml</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cerveja Puro Malte Stella Artois Belgium Garrafa 600ml</t>
+          <t>Cerveja Puro Malte Pure Gold Stella Artois Lata 8x350ml</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Stella Garrafa 600ml</t>
+          <t>Pure Gold lata 350ml</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cerveja Pilsen Lager Premium Stella Artois Pack 6 Garrafas 330ml Cada</t>
+          <t>Cerveja Stella Artois Gold Pack 6 Long Neck 330ml Cada</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1557,22 +1583,46 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Cerveja Stella Artois lata 350ml</t>
+          <t>Cerveja Puro Malte Stella Artois Belgium Garrafa 600ml</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Stella lata 350ml</t>
+          <t>Stella Garrafa 600ml</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Cerveja Pilsen Lager Premium Stella Artois Pack 6 Garrafas 330ml Cada</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Stella LN 330ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Cerveja Stella Artois lata 350ml</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Stella lata 350ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Cerveja Stella Artois long neck 330ml</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Stella LN 330ml</t>
         </is>

</xml_diff>